<commit_message>
Atualizando demais preços 12/06
</commit_message>
<xml_diff>
--- a/data/ProdutosFomatodos.xlsx
+++ b/data/ProdutosFomatodos.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="5"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="promoçoes"/>
@@ -3407,7 +3407,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3419,6 +3419,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFffffff"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -3505,7 +3511,7 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -6070,7 +6076,7 @@
         <v>10</v>
       </c>
       <c r="G20" s="4">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
@@ -12958,7 +12964,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="6" width="30.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="35.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="37.57642857142857" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="7" width="12.005" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="7" width="15.005" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="6" width="15.005" customWidth="1" bestFit="1"/>
@@ -14044,7 +14050,7 @@
         <v>10</v>
       </c>
       <c r="G47" s="4">
-        <v>200</v>
+        <v>203.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
@@ -14113,7 +14119,7 @@
         <v>10</v>
       </c>
       <c r="G50" s="4">
-        <v>377</v>
+        <v>378.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
@@ -14159,7 +14165,7 @@
         <v>10</v>
       </c>
       <c r="G52" s="4">
-        <v>377</v>
+        <v>378.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
@@ -14228,7 +14234,7 @@
         <v>10</v>
       </c>
       <c r="G55" s="4">
-        <v>377</v>
+        <v>378.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
@@ -14297,7 +14303,7 @@
         <v>10</v>
       </c>
       <c r="G58" s="4">
-        <v>377</v>
+        <v>378.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
@@ -14320,7 +14326,7 @@
         <v>10</v>
       </c>
       <c r="G59" s="4">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
@@ -14389,7 +14395,7 @@
         <v>10</v>
       </c>
       <c r="G62" s="4">
-        <v>392</v>
+        <v>393.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
@@ -14412,7 +14418,7 @@
         <v>10</v>
       </c>
       <c r="G63" s="4">
-        <v>372</v>
+        <v>373.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
@@ -14481,7 +14487,7 @@
         <v>10</v>
       </c>
       <c r="G66" s="4">
-        <v>262</v>
+        <v>263.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
@@ -19306,7 +19312,7 @@
         <v>10</v>
       </c>
       <c r="G3" s="4">
-        <v>15.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
@@ -19352,7 +19358,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="4">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
@@ -19421,7 +19427,7 @@
         <v>10</v>
       </c>
       <c r="G8" s="5">
-        <v>14.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
@@ -19467,7 +19473,7 @@
         <v>10</v>
       </c>
       <c r="G10" s="5">
-        <v>14.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
@@ -19513,7 +19519,7 @@
         <v>156</v>
       </c>
       <c r="G12" s="5">
-        <v>14.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
@@ -20873,7 +20879,7 @@
         <v>64.5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="19.5">
       <c r="A72" s="3" t="s">
         <v>822</v>
       </c>
@@ -20896,7 +20902,7 @@
         <v>300</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="19.5">
       <c r="A73" s="3" t="s">
         <v>822</v>
       </c>
@@ -20919,7 +20925,7 @@
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="19.5">
       <c r="A74" s="3" t="s">
         <v>824</v>
       </c>
@@ -20942,7 +20948,7 @@
         <v>180</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="19.5">
       <c r="A75" s="3" t="s">
         <v>824</v>
       </c>
@@ -20965,7 +20971,7 @@
         <v>38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="19.5">
       <c r="A76" s="3" t="s">
         <v>826</v>
       </c>
@@ -20988,7 +20994,7 @@
         <v>192.5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="19.5">
       <c r="A77" s="3" t="s">
         <v>826</v>
       </c>
@@ -21011,7 +21017,7 @@
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="19.5">
       <c r="A78" s="3" t="s">
         <v>826</v>
       </c>
@@ -21034,7 +21040,7 @@
         <v>43.5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="19.5">
       <c r="A79" s="3" t="s">
         <v>828</v>
       </c>
@@ -21057,7 +21063,7 @@
         <v>626</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="19.5">
       <c r="A80" s="3" t="s">
         <v>828</v>
       </c>
@@ -21080,7 +21086,7 @@
         <v>313</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="19.5">
       <c r="A81" s="3" t="s">
         <v>828</v>
       </c>
@@ -21103,7 +21109,7 @@
         <v>71</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="19.5">
       <c r="A82" s="3" t="s">
         <v>830</v>
       </c>
@@ -21126,7 +21132,7 @@
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="19.5">
       <c r="A83" s="3" t="s">
         <v>832</v>
       </c>
@@ -21149,7 +21155,7 @@
         <v>182</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="19.5">
       <c r="A84" s="3" t="s">
         <v>832</v>
       </c>
@@ -21172,7 +21178,7 @@
         <v>350</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="19.5">
       <c r="A85" s="3" t="s">
         <v>832</v>
       </c>
@@ -21195,7 +21201,7 @@
         <v>700</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="19.5">
       <c r="A86" s="3" t="s">
         <v>832</v>
       </c>
@@ -21218,7 +21224,7 @@
         <v>106</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="19.5">
       <c r="A87" s="3" t="s">
         <v>834</v>
       </c>
@@ -21241,7 +21247,7 @@
         <v>87</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="19.5">
       <c r="A88" s="3" t="s">
         <v>836</v>
       </c>
@@ -21264,7 +21270,7 @@
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="19.5">
       <c r="A89" s="3" t="s">
         <v>838</v>
       </c>
@@ -21287,7 +21293,7 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="19.5">
       <c r="A90" s="3" t="s">
         <v>840</v>
       </c>
@@ -21310,7 +21316,7 @@
         <v>119</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="19.5">
       <c r="A91" s="3" t="s">
         <v>840</v>
       </c>
@@ -21333,7 +21339,7 @@
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="19.5">
       <c r="A92" s="3" t="s">
         <v>840</v>
       </c>
@@ -21356,7 +21362,7 @@
         <v>228</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="19.5">
       <c r="A93" s="3" t="s">
         <v>842</v>
       </c>
@@ -21379,7 +21385,7 @@
         <v>125</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="19.5">
       <c r="A94" s="3" t="s">
         <v>842</v>
       </c>
@@ -22639,7 +22645,7 @@
         <v>10</v>
       </c>
       <c r="G15" s="5">
-        <v>94.5</v>
+        <v>95.5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">

</xml_diff>